<commit_message>
updates based on reviewer feedback
</commit_message>
<xml_diff>
--- a/mnp_compass/data/crosswalk.xlsx
+++ b/mnp_compass/data/crosswalk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\methods_navigator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\mnp_compass\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED35BA5A-C0B1-4113-AA0C-36BEA9D69899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1808C267-AF69-4D68-9FB5-98F8F4FD5257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5208,7 +5208,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5483,14 +5483,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5512,40 +5545,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="26" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6464,75 +6463,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:54" ht="66.599999999999994" hidden="1" customHeight="1">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="109" t="s">
+      <c r="B1" s="100"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="108"/>
-      <c r="N1" s="111" t="s">
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="102"/>
+      <c r="N1" s="105" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="98"/>
+      <c r="O1" s="106"/>
       <c r="P1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Q1" s="112" t="s">
+      <c r="Q1" s="107" t="s">
         <v>40</v>
       </c>
-      <c r="R1" s="97"/>
-      <c r="S1" s="97"/>
-      <c r="T1" s="97"/>
-      <c r="U1" s="97"/>
-      <c r="V1" s="97"/>
-      <c r="W1" s="97"/>
-      <c r="X1" s="97"/>
-      <c r="Y1" s="97"/>
-      <c r="Z1" s="97"/>
-      <c r="AA1" s="97"/>
-      <c r="AB1" s="97"/>
-      <c r="AC1" s="97"/>
-      <c r="AD1" s="98"/>
-      <c r="AE1" s="113" t="s">
+      <c r="R1" s="101"/>
+      <c r="S1" s="101"/>
+      <c r="T1" s="101"/>
+      <c r="U1" s="101"/>
+      <c r="V1" s="101"/>
+      <c r="W1" s="101"/>
+      <c r="X1" s="101"/>
+      <c r="Y1" s="101"/>
+      <c r="Z1" s="101"/>
+      <c r="AA1" s="101"/>
+      <c r="AB1" s="101"/>
+      <c r="AC1" s="101"/>
+      <c r="AD1" s="106"/>
+      <c r="AE1" s="108" t="s">
         <v>41</v>
       </c>
-      <c r="AF1" s="98"/>
-      <c r="AG1" s="96" t="s">
+      <c r="AF1" s="106"/>
+      <c r="AG1" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="AH1" s="97"/>
-      <c r="AI1" s="97"/>
-      <c r="AJ1" s="98"/>
+      <c r="AH1" s="101"/>
+      <c r="AI1" s="101"/>
+      <c r="AJ1" s="106"/>
       <c r="AK1" s="15"/>
       <c r="AL1" s="16" t="s">
         <v>43</v>
       </c>
       <c r="AM1" s="78"/>
-      <c r="AN1" s="99" t="s">
+      <c r="AN1" s="110" t="s">
         <v>44</v>
       </c>
-      <c r="AO1" s="98"/>
-      <c r="AP1" s="100" t="s">
+      <c r="AO1" s="106"/>
+      <c r="AP1" s="111" t="s">
         <v>45</v>
       </c>
-      <c r="AQ1" s="98"/>
-      <c r="AR1" s="101" t="s">
+      <c r="AQ1" s="106"/>
+      <c r="AR1" s="112" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" s="102"/>
-      <c r="AT1" s="102"/>
-      <c r="AU1" s="102"/>
+      <c r="AS1" s="113"/>
+      <c r="AT1" s="113"/>
+      <c r="AU1" s="113"/>
       <c r="AV1" s="17" t="s">
         <v>44</v>
       </c>
@@ -6541,11 +6540,11 @@
       </c>
       <c r="AX1" s="19"/>
       <c r="AY1" s="19"/>
-      <c r="AZ1" s="103" t="s">
+      <c r="AZ1" s="114" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" s="104"/>
-      <c r="BB1" s="105"/>
+      <c r="BA1" s="115"/>
+      <c r="BB1" s="116"/>
     </row>
     <row r="2" spans="1:54" s="4" customFormat="1" ht="57.75" customHeight="1">
       <c r="A2" s="20" t="s">
@@ -9477,7 +9476,9 @@
       <c r="AE31" s="47">
         <v>1</v>
       </c>
-      <c r="AF31" s="47"/>
+      <c r="AF31" s="47">
+        <v>1</v>
+      </c>
       <c r="AG31" s="47">
         <v>1</v>
       </c>
@@ -11255,7 +11256,9 @@
       <c r="AC49" s="47"/>
       <c r="AD49" s="47"/>
       <c r="AE49" s="47"/>
-      <c r="AF49" s="47"/>
+      <c r="AF49" s="47">
+        <v>3</v>
+      </c>
       <c r="AG49" s="47">
         <v>3</v>
       </c>
@@ -23248,7 +23251,9 @@
       <c r="AE176" s="82">
         <v>1</v>
       </c>
-      <c r="AF176" s="82"/>
+      <c r="AF176" s="82">
+        <v>1</v>
+      </c>
       <c r="AG176" s="82">
         <v>1</v>
       </c>
@@ -24663,7 +24668,7 @@
       <c r="B191" s="3" t="s">
         <v>1458</v>
       </c>
-      <c r="C191" s="115">
+      <c r="C191" s="83">
         <v>2026</v>
       </c>
       <c r="D191" s="3" t="s">
@@ -24755,7 +24760,7 @@
       <c r="B192" s="3" t="s">
         <v>1464</v>
       </c>
-      <c r="C192" s="115">
+      <c r="C192" s="83">
         <v>2026</v>
       </c>
       <c r="D192" s="3" t="s">
@@ -24839,17 +24844,17 @@
     <row r="193" spans="1:54" ht="14.3" customHeight="1">
       <c r="A193" s="70"/>
       <c r="B193" s="3"/>
-      <c r="C193" s="115"/>
+      <c r="C193" s="83"/>
       <c r="D193" s="3"/>
       <c r="E193" s="3"/>
       <c r="F193" s="68"/>
       <c r="G193" s="90"/>
-      <c r="H193" s="114"/>
-      <c r="I193" s="116"/>
+      <c r="H193" s="96"/>
+      <c r="I193" s="97"/>
       <c r="J193" s="81"/>
       <c r="K193" s="91"/>
       <c r="L193" s="83"/>
-      <c r="M193" s="117"/>
+      <c r="M193" s="98"/>
       <c r="N193" s="82"/>
       <c r="O193" s="82"/>
       <c r="P193" s="82"/>
@@ -28191,16 +28196,16 @@
     <row r="1018" spans="1:49" ht="14.3" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AR1:AU1"/>
+    <mergeCell ref="AZ1:BB1"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="F1:M1"/>
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="Q1:AD1"/>
     <mergeCell ref="AE1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AR1:AU1"/>
-    <mergeCell ref="AZ1:BB1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E144" r:id="rId1" xr:uid="{A81C656A-0A99-4267-9649-0EEFD2B27222}"/>

</xml_diff>

<commit_message>
added a few air references
</commit_message>
<xml_diff>
--- a/mnp_compass/data/crosswalk.xlsx
+++ b/mnp_compass/data/crosswalk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\mnp_compass\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1808C267-AF69-4D68-9FB5-98F8F4FD5257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7451A300-0E7C-401C-97B1-CB39302905A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Reviewer" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Crosswalk Table'!$A$2:$BB$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Crosswalk Table'!$A$2:$BB$196</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2707" uniqueCount="1468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="1490">
   <si>
     <t>Reviewer Name</t>
   </si>
@@ -4647,6 +4647,75 @@
   </si>
   <si>
     <t>Review of 58 active standards were identified on Standards Australia International Global database</t>
+  </si>
+  <si>
+    <t>ISO/AWI 26731</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.iso.org/standard/94332.html </t>
+  </si>
+  <si>
+    <t>ISO/AWI 26731: Spectroscopic Method for Measurement of Microplastics in Air</t>
+  </si>
+  <si>
+    <t>Under Development as of 10-23-2026</t>
+  </si>
+  <si>
+    <t>This document provides the scope and basic principles for a standardized method for the quantitative analysis and characterization of microplastics (MPs) in air. It establishes a consistent procedural framework covering the entire analytical process, from sampling to pretreatment, analysis, quantification, and characterization of airborne MPs. This document addresses the collection of air samples using low- or high-volume samplers, recovery and pretreatment of samples using metal filters, and the determination of the number, size, shape, and polymer type of MPs by means of vibrational spectroscopic techniques (e.g., μ-FTIR or μ-Raman) coupled with an image processing system equipped with a microscope. The standardized approach aims to improve the reliability, reproducibility, and comparability of measurement results obtained by different laboratories and studies. This document applies to the analysis of ambient air, recognizing that MPs can be present as a result of atmospheric transport, deposition, and resuspension and may coexist with particulate matters. It supports the generation of harmonized data for environmental monitoring of airborne MPs and the assessment of their potential impacts on human health and the environment. This document is applicable to: a) research institutes, testing and inspection laboratories, and academic bodies conducting quantitative and qualitative analyses of MPs in air; b) governmental and public authorities involved in air quality management, environmental monitoring, and risk assessment related to airborne MPs; c) industries and service providers engaged in the development of analytical instruments or managemental technologies for MPs in air.</t>
+  </si>
+  <si>
+    <t>ASTM WK94202</t>
+  </si>
+  <si>
+    <t>ASTM WK94202: New Test Method for Direct Analysis of Airborne Microplastics (MP) Collected on Quartz Particulate Matter (PM) Filters by Pyrolysis-Gas Chromatography/Mass Spectrometry (Py-GC/MS)</t>
+  </si>
+  <si>
+    <t>https://www.astm.org/membership-participation/technical-committees/workitems/workitem-wk94202</t>
+  </si>
+  <si>
+    <t>The proposed standard is intended to provide a standardized method to identify and quantify the mass of 11 target polymer types from quartz PM air filters. The proposed method includes standard procedures for sample collection and handling, calibration, method validation, data quality objectives, and analysis of target polymer types in quartz PM air filters using analytical pyrolysis-gas chromatography/mass spectrometry (Py-GC/MS).</t>
+  </si>
+  <si>
+    <t>Aves et al., 2026</t>
+  </si>
+  <si>
+    <t>Comparative assessment of five analytical methods for airborne microplastics highlights importance of identifying sub-
+μ
+ methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nature.com/articles/s41598-026-49405-2 </t>
+  </si>
+  <si>
+    <t>Microplastics are an emerging class of contaminants that are widespread in the environment. While studies on airborne microplastics are rapidly increasing, the lack of standardised sampling and analysis methods is hindering progress towards accurately quantifying their global distribution. This study used existing analytical methodologies to understand the variability in identifying and quantifying airborne microplastics. High-volume aerosol samples were collected at a remote site in New Zealand and were analysed by micro-Fourier transform infrared spectroscopy, micro-Raman spectroscopy, Nile red staining combined with fluorescence microscopy, pyrolysis-gas chromatography/mass spectrometry and thermal desorption-proton transfer reaction-mass spectrometry, with all methods reporting different concentrations and polymer types. No particles were larger than 100 µm, and 98% of particles were smaller than 10 µm, highlighting the importance of methods that can analyse sub-10 µm particles. This study highlights the need for caution when comparing airborne microplastic datasets analysed using different methods.</t>
+  </si>
+  <si>
+    <t>Microplastics (&lt;10 um)</t>
+  </si>
+  <si>
+    <t>Method comparison study on controlled samples</t>
+  </si>
+  <si>
+    <t>µFTIR; µRaman; Py-GC-MS; Nile red</t>
+  </si>
+  <si>
+    <t>https://std.samr.gov.cn/gb/search/gbDetailed?id=49FD1852C85FC31FE06397BE0A0A1304</t>
+  </si>
+  <si>
+    <t>China Petroleum and Chemical Industry Federation (2026)</t>
+  </si>
+  <si>
+    <t>Determination of five resin microplastics, including polyethylene, in ambient air using pyrolysis-thermal desorption-gas chromatography-mass spectrometry.</t>
+  </si>
+  <si>
+    <t>Initiated 2026-01-28; 18 month cycle</t>
+  </si>
+  <si>
+    <t>Under development as of 10-23-2026</t>
+  </si>
+  <si>
+    <t>The national standard project, "Determination of Five Resin Microplastics, Including Polyethylene, in Ambient Air: Thermochemical Desorption-Gas Chromatography-Mass Spectrometry," is under the jurisdiction of TC15 (National Technical Committee on Plastics Standardization) and implemented by TC15SC14 (Recycling and Environment Subcommittee of the National Technical Committee on Plastics Standardization). The competent authority is the China Petroleum and Chemical Industry Federation .
+The main drafting units include Zhejiang Normal University and Guangzhou Institute of Quality Inspection .</t>
   </si>
 </sst>
 </file>
@@ -4841,7 +4910,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4970,14 +5039,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4EAFB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="19">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -5181,34 +5244,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC6C6C6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5483,47 +5524,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="26" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5546,6 +5554,31 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6065,8 +6098,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}" name="Table2" displayName="Table2" ref="A2:BB193" totalsRowShown="0" headerRowBorderDxfId="51">
-  <autoFilter ref="A2:BB193" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}" name="Table2" displayName="Table2" ref="A2:BB196" totalsRowShown="0" headerRowBorderDxfId="51">
+  <autoFilter ref="A2:BB196" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:BB176">
     <sortCondition ref="A2:A176"/>
   </sortState>
@@ -6463,75 +6496,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:54" ht="66.599999999999994" hidden="1" customHeight="1">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="103" t="s">
+      <c r="B1" s="107"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="104"/>
-      <c r="J1" s="104"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="100"/>
-      <c r="M1" s="102"/>
-      <c r="N1" s="105" t="s">
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="106"/>
+      <c r="O1" s="98"/>
       <c r="P1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Q1" s="107" t="s">
+      <c r="Q1" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="101"/>
-      <c r="U1" s="101"/>
-      <c r="V1" s="101"/>
-      <c r="W1" s="101"/>
-      <c r="X1" s="101"/>
-      <c r="Y1" s="101"/>
-      <c r="Z1" s="101"/>
-      <c r="AA1" s="101"/>
-      <c r="AB1" s="101"/>
-      <c r="AC1" s="101"/>
-      <c r="AD1" s="106"/>
-      <c r="AE1" s="108" t="s">
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="98"/>
+      <c r="AE1" s="113" t="s">
         <v>41</v>
       </c>
-      <c r="AF1" s="106"/>
-      <c r="AG1" s="109" t="s">
+      <c r="AF1" s="98"/>
+      <c r="AG1" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="AH1" s="101"/>
-      <c r="AI1" s="101"/>
-      <c r="AJ1" s="106"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="98"/>
       <c r="AK1" s="15"/>
       <c r="AL1" s="16" t="s">
         <v>43</v>
       </c>
       <c r="AM1" s="78"/>
-      <c r="AN1" s="110" t="s">
+      <c r="AN1" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="AO1" s="106"/>
-      <c r="AP1" s="111" t="s">
+      <c r="AO1" s="98"/>
+      <c r="AP1" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="AQ1" s="106"/>
-      <c r="AR1" s="112" t="s">
+      <c r="AQ1" s="98"/>
+      <c r="AR1" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" s="113"/>
-      <c r="AT1" s="113"/>
-      <c r="AU1" s="113"/>
+      <c r="AS1" s="102"/>
+      <c r="AT1" s="102"/>
+      <c r="AU1" s="102"/>
       <c r="AV1" s="17" t="s">
         <v>44</v>
       </c>
@@ -6540,11 +6573,11 @@
       </c>
       <c r="AX1" s="19"/>
       <c r="AY1" s="19"/>
-      <c r="AZ1" s="114" t="s">
+      <c r="AZ1" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" s="115"/>
-      <c r="BB1" s="116"/>
+      <c r="BA1" s="104"/>
+      <c r="BB1" s="105"/>
     </row>
     <row r="2" spans="1:54" s="4" customFormat="1" ht="57.75" customHeight="1">
       <c r="A2" s="20" t="s">
@@ -24842,22 +24875,50 @@
       </c>
     </row>
     <row r="193" spans="1:54" ht="14.3" customHeight="1">
-      <c r="A193" s="70"/>
-      <c r="B193" s="3"/>
-      <c r="C193" s="83"/>
-      <c r="D193" s="3"/>
-      <c r="E193" s="3"/>
-      <c r="F193" s="68"/>
-      <c r="G193" s="90"/>
-      <c r="H193" s="96"/>
-      <c r="I193" s="97"/>
-      <c r="J193" s="81"/>
-      <c r="K193" s="91"/>
-      <c r="L193" s="83"/>
-      <c r="M193" s="98"/>
+      <c r="A193" s="70">
+        <v>192</v>
+      </c>
+      <c r="B193" s="3" t="s">
+        <v>1468</v>
+      </c>
+      <c r="C193" s="83">
+        <v>2026</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>1470</v>
+      </c>
+      <c r="E193" s="89" t="s">
+        <v>1469</v>
+      </c>
+      <c r="F193" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="G193" s="40" t="s">
+        <v>697</v>
+      </c>
+      <c r="H193" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="I193" s="74" t="s">
+        <v>105</v>
+      </c>
+      <c r="J193" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="K193" s="91" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L193" s="83" t="s">
+        <v>1399</v>
+      </c>
+      <c r="M193" s="85" t="s">
+        <v>186</v>
+      </c>
       <c r="N193" s="82"/>
       <c r="O193" s="82"/>
-      <c r="P193" s="82"/>
+      <c r="P193" s="82">
+        <v>2</v>
+      </c>
       <c r="Q193" s="82"/>
       <c r="R193" s="82"/>
       <c r="S193" s="82"/>
@@ -24869,45 +24930,350 @@
       <c r="Y193" s="82"/>
       <c r="Z193" s="82"/>
       <c r="AA193" s="82"/>
-      <c r="AB193" s="82"/>
+      <c r="AB193" s="82">
+        <v>2</v>
+      </c>
       <c r="AC193" s="82"/>
       <c r="AD193" s="82"/>
-      <c r="AE193" s="82"/>
-      <c r="AF193" s="82"/>
-      <c r="AG193" s="82"/>
-      <c r="AH193" s="82"/>
-      <c r="AI193" s="82"/>
+      <c r="AE193" s="82">
+        <v>2</v>
+      </c>
+      <c r="AF193" s="82">
+        <v>2</v>
+      </c>
+      <c r="AG193" s="82">
+        <v>2</v>
+      </c>
+      <c r="AH193" s="82">
+        <v>2</v>
+      </c>
+      <c r="AI193" s="82">
+        <v>2</v>
+      </c>
       <c r="AJ193" s="82"/>
       <c r="AK193" s="82"/>
       <c r="AL193" s="82"/>
       <c r="AM193" s="82"/>
-      <c r="AN193" s="82"/>
-      <c r="AO193" s="67"/>
-      <c r="AP193" s="82"/>
+      <c r="AN193" s="82">
+        <v>2</v>
+      </c>
+      <c r="AO193" s="67">
+        <v>2</v>
+      </c>
+      <c r="AP193" s="82">
+        <v>2</v>
+      </c>
       <c r="AQ193" s="82"/>
       <c r="AR193" s="82"/>
       <c r="AS193" s="82"/>
       <c r="AT193" s="67"/>
       <c r="AU193" s="82"/>
       <c r="AV193" s="82"/>
-      <c r="AW193" s="10"/>
+      <c r="AW193" s="10" t="s">
+        <v>1471</v>
+      </c>
       <c r="AX193" s="83"/>
-      <c r="AY193" s="83"/>
-      <c r="AZ193" s="10"/>
+      <c r="AY193" s="83" t="s">
+        <v>1471</v>
+      </c>
+      <c r="AZ193" s="10" t="s">
+        <v>1393</v>
+      </c>
       <c r="BA193" s="45"/>
-      <c r="BB193" s="10"/>
+      <c r="BB193" s="10" t="s">
+        <v>1472</v>
+      </c>
     </row>
     <row r="194" spans="1:54" ht="14.3" customHeight="1">
-      <c r="A194" s="70"/>
-      <c r="AW194" s="10"/>
+      <c r="A194" s="70">
+        <v>193</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C194" s="114">
+        <v>2025</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>1474</v>
+      </c>
+      <c r="E194" s="89" t="s">
+        <v>1475</v>
+      </c>
+      <c r="F194" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="G194" s="40" t="s">
+        <v>697</v>
+      </c>
+      <c r="H194" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="I194" s="74" t="s">
+        <v>105</v>
+      </c>
+      <c r="J194" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="K194" s="91" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L194" s="83" t="s">
+        <v>1399</v>
+      </c>
+      <c r="M194" s="85" t="s">
+        <v>186</v>
+      </c>
+      <c r="N194" s="82"/>
+      <c r="O194" s="82"/>
+      <c r="P194" s="82">
+        <v>2</v>
+      </c>
+      <c r="Q194" s="82"/>
+      <c r="R194" s="82"/>
+      <c r="S194" s="82"/>
+      <c r="T194" s="82"/>
+      <c r="U194" s="82"/>
+      <c r="V194" s="82"/>
+      <c r="W194" s="82"/>
+      <c r="X194" s="82"/>
+      <c r="Y194" s="82"/>
+      <c r="Z194" s="82"/>
+      <c r="AA194" s="82"/>
+      <c r="AB194" s="82">
+        <v>2</v>
+      </c>
+      <c r="AC194" s="82"/>
+      <c r="AD194" s="82"/>
+      <c r="AE194" s="82">
+        <v>2</v>
+      </c>
+      <c r="AF194" s="82"/>
+      <c r="AG194" s="82">
+        <v>5</v>
+      </c>
+      <c r="AH194" s="82"/>
+      <c r="AI194" s="82"/>
+      <c r="AJ194" s="82">
+        <v>2</v>
+      </c>
+      <c r="AK194" s="82"/>
+      <c r="AL194" s="82"/>
+      <c r="AM194" s="82"/>
+      <c r="AN194" s="82"/>
+      <c r="AO194" s="67">
+        <v>2</v>
+      </c>
+      <c r="AP194" s="82">
+        <v>2</v>
+      </c>
+      <c r="AQ194" s="82"/>
+      <c r="AR194" s="82"/>
+      <c r="AS194" s="82"/>
+      <c r="AT194" s="67"/>
+      <c r="AU194" s="82"/>
+      <c r="AV194" s="82"/>
+      <c r="AW194" s="10" t="s">
+        <v>1471</v>
+      </c>
+      <c r="AX194" s="83"/>
+      <c r="AY194" s="83" t="s">
+        <v>1471</v>
+      </c>
+      <c r="AZ194" s="10" t="s">
+        <v>1393</v>
+      </c>
+      <c r="BA194" s="45"/>
+      <c r="BB194" s="10" t="s">
+        <v>1476</v>
+      </c>
     </row>
     <row r="195" spans="1:54" ht="14.3" customHeight="1">
-      <c r="A195" s="70"/>
-      <c r="AW195" s="10"/>
+      <c r="A195" s="70">
+        <v>194</v>
+      </c>
+      <c r="B195" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C195" s="114">
+        <v>2026</v>
+      </c>
+      <c r="D195" s="10" t="s">
+        <v>1478</v>
+      </c>
+      <c r="E195" s="89" t="s">
+        <v>1479</v>
+      </c>
+      <c r="F195" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="G195" s="40" t="s">
+        <v>697</v>
+      </c>
+      <c r="H195" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="I195" s="77" t="s">
+        <v>240</v>
+      </c>
+      <c r="J195" s="41" t="s">
+        <v>1483</v>
+      </c>
+      <c r="K195" s="91" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L195" s="83" t="s">
+        <v>1399</v>
+      </c>
+      <c r="M195" s="85" t="s">
+        <v>186</v>
+      </c>
+      <c r="N195" s="82"/>
+      <c r="O195" s="82"/>
+      <c r="P195" s="82"/>
+      <c r="Q195" s="82"/>
+      <c r="R195" s="82"/>
+      <c r="S195" s="82"/>
+      <c r="T195" s="82"/>
+      <c r="U195" s="82"/>
+      <c r="V195" s="82"/>
+      <c r="W195" s="82"/>
+      <c r="X195" s="82"/>
+      <c r="Y195" s="82"/>
+      <c r="Z195" s="82"/>
+      <c r="AA195" s="82"/>
+      <c r="AB195" s="82">
+        <v>3</v>
+      </c>
+      <c r="AC195" s="82"/>
+      <c r="AD195" s="82"/>
+      <c r="AE195" s="82"/>
+      <c r="AF195" s="82"/>
+      <c r="AG195" s="82"/>
+      <c r="AH195" s="82">
+        <v>3</v>
+      </c>
+      <c r="AI195" s="82">
+        <v>3</v>
+      </c>
+      <c r="AJ195" s="82"/>
+      <c r="AK195" s="82"/>
+      <c r="AL195" s="82"/>
+      <c r="AM195" s="82"/>
+      <c r="AN195" s="82"/>
+      <c r="AO195" s="67"/>
+      <c r="AP195" s="82"/>
+      <c r="AQ195" s="82"/>
+      <c r="AR195" s="82"/>
+      <c r="AS195" s="82"/>
+      <c r="AT195" s="67"/>
+      <c r="AU195" s="82"/>
+      <c r="AV195" s="82"/>
+      <c r="AW195" s="10" t="s">
+        <v>1482</v>
+      </c>
+      <c r="AX195" s="83"/>
+      <c r="AY195" s="83"/>
+      <c r="AZ195" s="10" t="s">
+        <v>1481</v>
+      </c>
+      <c r="BA195" s="45"/>
+      <c r="BB195" s="10" t="s">
+        <v>1480</v>
+      </c>
     </row>
     <row r="196" spans="1:54" ht="14.3" customHeight="1">
-      <c r="A196" s="70"/>
-      <c r="AW196" s="10"/>
+      <c r="A196" s="70">
+        <v>195</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C196" s="114">
+        <v>2026</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>1486</v>
+      </c>
+      <c r="E196" s="89" t="s">
+        <v>1484</v>
+      </c>
+      <c r="F196" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="G196" s="40" t="s">
+        <v>697</v>
+      </c>
+      <c r="H196" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="I196" s="74" t="s">
+        <v>105</v>
+      </c>
+      <c r="J196" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="K196" s="91" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L196" s="83" t="s">
+        <v>1399</v>
+      </c>
+      <c r="M196" s="85" t="s">
+        <v>186</v>
+      </c>
+      <c r="N196" s="82"/>
+      <c r="O196" s="82"/>
+      <c r="P196" s="82"/>
+      <c r="Q196" s="82"/>
+      <c r="R196" s="82"/>
+      <c r="S196" s="82"/>
+      <c r="T196" s="82"/>
+      <c r="U196" s="82"/>
+      <c r="V196" s="82"/>
+      <c r="W196" s="82"/>
+      <c r="X196" s="82"/>
+      <c r="Y196" s="82"/>
+      <c r="Z196" s="82"/>
+      <c r="AA196" s="82"/>
+      <c r="AB196" s="82">
+        <v>2</v>
+      </c>
+      <c r="AC196" s="82"/>
+      <c r="AD196" s="82"/>
+      <c r="AE196" s="82"/>
+      <c r="AF196" s="82"/>
+      <c r="AG196" s="82"/>
+      <c r="AH196" s="82"/>
+      <c r="AI196" s="82"/>
+      <c r="AJ196" s="82">
+        <v>2</v>
+      </c>
+      <c r="AK196" s="82"/>
+      <c r="AL196" s="82"/>
+      <c r="AM196" s="82"/>
+      <c r="AN196" s="82"/>
+      <c r="AO196" s="67"/>
+      <c r="AP196" s="82"/>
+      <c r="AQ196" s="82"/>
+      <c r="AR196" s="82"/>
+      <c r="AS196" s="82"/>
+      <c r="AT196" s="67"/>
+      <c r="AU196" s="82"/>
+      <c r="AV196" s="82"/>
+      <c r="AW196" s="10" t="s">
+        <v>1487</v>
+      </c>
+      <c r="AY196" s="83" t="s">
+        <v>1488</v>
+      </c>
+      <c r="AZ196" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="BA196" s="45"/>
+      <c r="BB196" s="10" t="s">
+        <v>1489</v>
+      </c>
     </row>
     <row r="197" spans="1:54" ht="14.3" customHeight="1">
       <c r="A197" s="70"/>
@@ -28196,16 +28562,16 @@
     <row r="1018" spans="1:49" ht="14.3" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="Q1:AD1"/>
+    <mergeCell ref="AE1:AF1"/>
     <mergeCell ref="AG1:AJ1"/>
     <mergeCell ref="AN1:AO1"/>
     <mergeCell ref="AP1:AQ1"/>
     <mergeCell ref="AR1:AU1"/>
     <mergeCell ref="AZ1:BB1"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="Q1:AD1"/>
-    <mergeCell ref="AE1:AF1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E144" r:id="rId1" xr:uid="{A81C656A-0A99-4267-9649-0EEFD2B27222}"/>
@@ -28222,11 +28588,15 @@
     <hyperlink ref="E190" r:id="rId12" xr:uid="{8048047A-11A2-4914-AA30-CADB42BA1A40}"/>
     <hyperlink ref="E191" r:id="rId13" display="https://doi.org/10.1016/j.envint.2026.110429" xr:uid="{A8CFEA85-96A6-4EB2-9519-3D355F9DB6A8}"/>
     <hyperlink ref="E192" r:id="rId14" xr:uid="{50B7E77B-853E-4D24-9D46-277F2F5E3E9E}"/>
+    <hyperlink ref="E193" r:id="rId15" xr:uid="{3A8E5899-9B40-4D28-B8E0-C96DB39D66E6}"/>
+    <hyperlink ref="E194" r:id="rId16" xr:uid="{4F449559-2314-4B52-A381-AEBCA7C6EF85}"/>
+    <hyperlink ref="E195" r:id="rId17" xr:uid="{F4590893-0990-4FE8-BB10-C3547466E697}"/>
+    <hyperlink ref="E196" r:id="rId18" xr:uid="{DE7ED8D7-ECEC-41DB-B080-ED092D78AE64}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId15"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId19"/>
   <tableParts count="1">
-    <tablePart r:id="rId16"/>
+    <tablePart r:id="rId20"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>